<commit_message>
Update project with final version and Docker
</commit_message>
<xml_diff>
--- a/sugar_desserts.xlsx
+++ b/sugar_desserts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Downloads\2026\Graduated project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B7A1ECC-5460-411D-99F3-7ADD1A9C7834}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26181C95-08E6-4ABA-A3C9-2D83E028B46C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{AD9B9CF5-758B-4BD4-B7F4-E995B4829E1B}"/>
   </bookViews>
@@ -123,9 +123,6 @@
     <t>stuffed pancake with nuts or cheese,soaked with syrup or honey</t>
   </si>
   <si>
-    <t>Halawa tehini</t>
-  </si>
-  <si>
     <t>Sugar_per_100g</t>
   </si>
   <si>
@@ -133,6 +130,9 @@
   </si>
   <si>
     <t>shortbread pastry stuffed with sweet date, walnut and pisachios</t>
+  </si>
+  <si>
+    <t>Halava tehini</t>
   </si>
 </sst>
 </file>
@@ -534,7 +534,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>1</v>
@@ -641,7 +641,7 @@
     </row>
     <row r="11" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B11">
         <v>30</v>
@@ -718,13 +718,13 @@
     </row>
     <row r="18" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B18">
         <v>12</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>